<commit_message>
cambio de nombre Epcoro -- Sinchy Wayra
</commit_message>
<xml_diff>
--- a/docs/hoja.xlsx
+++ b/docs/hoja.xlsx
@@ -111,7 +111,7 @@
     <t xml:space="preserve">CAJA DE SALUD APORTE 1,8%</t>
   </si>
   <si>
-    <t xml:space="preserve">si</t>
+    <t xml:space="preserve">no</t>
   </si>
   <si>
     <t xml:space="preserve">NOMBRE VENDEDOR</t>
@@ -690,9 +690,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2596320</xdr:colOff>
+      <xdr:colOff>2595960</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>188640</xdr:rowOff>
+      <xdr:rowOff>188280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -706,7 +706,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="459720" y="258480"/>
-          <a:ext cx="2337840" cy="621000"/>
+          <a:ext cx="2337480" cy="620640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -733,9 +733,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2596320</xdr:colOff>
+      <xdr:colOff>2595960</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>188640</xdr:rowOff>
+      <xdr:rowOff>188280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -749,7 +749,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="459720" y="258480"/>
-          <a:ext cx="2337840" cy="621000"/>
+          <a:ext cx="2337480" cy="620640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1061,7 +1061,7 @@
       <c r="I4" s="8"/>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="21.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="F11" s="21" t="n">
         <f aca="false">F10*H11</f>
-        <v>20329.4047172837</v>
+        <v>0</v>
       </c>
       <c r="G11" s="13"/>
       <c r="H11" s="22" t="n">
         <f aca="false">IF(C20="NO",0,0.018)</f>
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="I11" s="23"/>
       <c r="J11" s="7"/>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="F12" s="21" t="n">
         <f aca="false">F10-F11</f>
-        <v>1109081.96846515</v>
+        <v>1129411.37318243</v>
       </c>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
@@ -1767,7 +1767,7 @@
       <c r="I4" s="8"/>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="21.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>

</xml_diff>